<commit_message>
Add Norm Ai to week ending 10-Jul-26 as RegTech (Financial Info & Analytics)
Per reviewer call, include Norm Ai ($120M Series C @ $1.2B, Khosla Ventures)
on the Raises tab as RegTech/compliance analytics rather than excluding it as
legal AI. Raises now 3 (Norm Ai, Super.com, EDX Markets).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U2wV75eD6i9VwECvq35RCT
</commit_message>
<xml_diff>
--- a/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-10.xlsx
+++ b/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-10.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All M&amp;A (PE &amp; Strategic)'!$A$1:$R$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$M$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$M$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1028,7 +1028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1231,11 +1231,71 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>10-Jul-26</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Financial Info &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>07-Jul-26</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Norm Ai</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Khosla Ventures</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>AI-native regulatory-compliance and legal-review platform deploying rules-trained agents for banks, insurers, asset managers and other regulated enterprises</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M3"/>
+  <autoFilter ref="A1:M4"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update week ending 10-Jul-26: add Norm AI (RegTech raise) and Nium/Cypher (Payments M&A)
After a deeper source reconciliation across FinTech Global, FinTech Futures,
This Week in Fintech, Finovate and regional press:
- Add Norm AI ($120M Series C @ $1.2B, Khosla) to Raises as Financial Info &
  Analytics (RegTech / regulatory-compliance AI).
- Add Nium -> Cypher (08-Jul, undisclosed) to M&A as Payments (crypto wallet /
  card-issuing tech acquisition).

Now 6 M&A + 3 raises. No other qualifying >=$25M raise or control-M&A surfaced
in-window; Nordic Capital/Liberis+Qred confirmed out of window (announced 18-Jun).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U2wV75eD6i9VwECvq35RCT
</commit_message>
<xml_diff>
--- a/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-10.xlsx
+++ b/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-10.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Growth Capital Raises" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All M&amp;A (PE &amp; Strategic)'!$A$1:$R$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All M&amp;A (PE &amp; Strategic)'!$A$1:$R$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$M$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1009,14 +1009,103 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>10-Jul-26</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Strategic M&amp;A</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>08-Jul-26</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Cypher</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Nium</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Crypto-native non-custodial wallet and card-issuing platform bridging fiat and on-chain money movement</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R6"/>
+  <autoFilter ref="A1:R7"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add ThrivePass/Shore Capital (PE Buyout) to week ending 10-Jul-26
ThrivePass (Denver employee-benefits platform: lifestyle spending accounts,
pre-tax benefits, COBRA, reimbursements) acquired by Shore Capital Partners,
announced 08-Jul-26 (BusinessWire). First PE Buyout of the week; borderline
benefits/HR-fintech included on the spending-account/money-movement core
(same basis as Warp/BIPO). Now 7 M&A + 3 raises.

Checked and excluded from the same batch: Alta $25M (GTM/sales SaaS, not
fintech), Mobeus->Assured Underwriting/ANV (traditional travel MGA, not
fintech), Bizay $55M (e-commerce marketplace, not fintech). Blipay/Tilt
confirmed out-of-window (announced 01-Jul).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U2wV75eD6i9VwECvq35RCT
</commit_message>
<xml_diff>
--- a/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-10.xlsx
+++ b/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-10.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Growth Capital Raises" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All M&amp;A (PE &amp; Strategic)'!$B$3:$R$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All M&amp;A (PE &amp; Strategic)'!$B$3:$R$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$3:$M$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:R9"/>
+  <dimension ref="A3:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.73" customWidth="1" min="1" max="1"/>
@@ -872,46 +872,52 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Corporate Financial Function</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Strategic M&amp;A</t>
+          <t>PE Buyout</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>07-Jul-26</t>
+          <t>08-Jul-26</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Círculo de Crédito</t>
+          <t>ThrivePass</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Equifax</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>750</v>
-      </c>
-      <c r="J7" s="6" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>12.1</v>
+          <t>Shore Capital Partners</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>Consumer credit bureau in Mexico providing credit reports, scores and risk analytics to lenders</t>
+          <t>Employee-benefits administration platform for lifestyle spending accounts, pre-tax benefits, COBRA and tuition reimbursement — HR-benefits tech with an embedded spending-account/money-movement layer</t>
         </is>
       </c>
       <c r="M7" s="8" t="inlineStr">
@@ -921,12 +927,12 @@
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>Equifax investor press release</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>LTM to 30-Jun-26 rev ~$134M (+31% YoY), adj. EBITDA ~$62M; EV $750M ($825M gross less ~$75M cash, no debt) -&gt; 5.6x rev / 12.1x EBITDA</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P7" s="4" t="inlineStr">
@@ -954,12 +960,12 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Financial Info &amp; Analytics</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -974,32 +980,26 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Send Technology Solutions</t>
+          <t>Círculo de Crédito</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Duck Creek Technologies</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K8" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Equifax</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>12.1</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
-          <t>AI-native underwriting orchestration engine for commercial, specialty, reinsurance and MGA/delegated-authority insurers</t>
+          <t>Consumer credit bureau in Mexico providing credit reports, scores and risk analytics to lenders</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr">
@@ -1009,12 +1009,12 @@
       </c>
       <c r="N8" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Equifax investor press release</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>LTM to 30-Jun-26 rev ~$134M (+31% YoY), adj. EBITDA ~$62M; EV $750M ($825M gross less ~$75M cash, no debt) -&gt; 5.6x rev / 12.1x EBITDA</t>
         </is>
       </c>
       <c r="P8" s="4" t="inlineStr">
@@ -1042,87 +1042,175 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
+          <t>InsurTech</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Strategic M&amp;A</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>07-Jul-26</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Send Technology Solutions</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Duck Creek Technologies</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>AI-native underwriting orchestration engine for commercial, specialty, reinsurance and MGA/delegated-authority insurers</t>
+        </is>
+      </c>
+      <c r="M9" s="8" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P9" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q9" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R9" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>10-Jul-26</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
           <t>Payments</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>Strategic M&amp;A</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>08-Jul-26</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Cypher</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>Nium</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K9" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L9" s="7" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
         <is>
           <t>Crypto-native non-custodial wallet and card-issuing platform bridging fiat and on-chain money movement</t>
         </is>
       </c>
-      <c r="M9" s="8" t="inlineStr">
+      <c r="M10" s="8" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="N9" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O9" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P9" s="4" t="inlineStr">
+      <c r="N10" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P10" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="Q9" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R9" s="4" t="inlineStr">
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R10" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B3:R9"/>
+  <autoFilter ref="B3:R10"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId2"/>
@@ -1130,6 +1218,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Kord (RE & Mortgage Tech raise) to week ending 10-Jul-26
Kord (UK, FCA-regulated) unifies identity/AML checks and client-money payment
processing for estate agents, conveyancers and law firms. £6.4M (~$8.6M)
Series A led by Guinness Ventures, announced 08-Jul-26. Added per direct
request with the $25M floor waived; passes all other criteria (in-window,
genuine payments/RegTech fintech core, credible sources, equity round).
Now 7 M&A + 4 raises.

HousApp (€4.3M) held out: announced 02-Jul (prior week) and is proptech
agent-CRM SaaS with no money-movement/financial core.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U2wV75eD6i9VwECvq35RCT
</commit_message>
<xml_diff>
--- a/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-10.xlsx
+++ b/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-10.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All M&amp;A (PE &amp; Strategic)'!$B$3:$R$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$3:$M$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$3:$M$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1230,7 +1230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:M6"/>
+  <dimension ref="A3:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.73" customWidth="1" min="1" max="1"/>
@@ -1492,12 +1492,74 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>10-Jul-26</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Real Estate &amp; Mortgage Tech</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>08-Jul-26</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Kord</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Guinness Ventures</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>FCA-regulated platform unifying identity/AML checks and client-money payment processing for estate agents, conveyancers and law firms</t>
+        </is>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:M6"/>
+  <autoFilter ref="A3:M7"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Skello, GoCharting, MountainSeed, BrightAnalytics to week ending 10-Jul-26
Four sponsor/requested deals, all in-window and vetted:
- BrightAnalytics (Belgium CFO/CPM software) -> M&A tab as PE Buyout: PSG
  Equity took a MAJORITY (control) stake (09-Jul), so it's not a raise.
- MountainSeed ($38M, Long Ridge minority, 09-Jul) -> Raises, Banking &
  Lending Tech (appraisal/valuation + capital-markets tech for banks/CUs).
- GoCharting (Long Ridge growth, size undisclosed/waived, 07-Jul, India) ->
  Raises, Capital Markets Tech (order-flow charting for traders).
- Skello (EUR200M ~$230M, Bridgepoint minority, 07-Jul, France) -> Raises,
  Corporate Financial Function. BORDERLINE: HR/workforce-scheduling with
  payroll prep; included per request but flagged as weakest fintech fit.

Now 8 M&A + 7 raises.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U2wV75eD6i9VwECvq35RCT
</commit_message>
<xml_diff>
--- a/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-10.xlsx
+++ b/weekly-deals/outputs/Weekly_Fintech_Deals_2026-07-10.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Growth Capital Raises" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All M&amp;A (PE &amp; Strategic)'!$B$3:$R$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$3:$M$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All M&amp;A (PE &amp; Strategic)'!$B$3:$R$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$3:$M$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:R10"/>
+  <dimension ref="A3:R11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.73" customWidth="1" min="1" max="1"/>
@@ -960,46 +960,52 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Corporate Financial Function</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Strategic M&amp;A</t>
+          <t>PE Buyout</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>07-Jul-26</t>
+          <t>09-Jul-26</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Círculo de Crédito</t>
+          <t>BrightAnalytics</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Equifax</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="n">
-        <v>750</v>
-      </c>
-      <c r="J8" s="6" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="K8" s="6" t="n">
-        <v>12.1</v>
+          <t>PSG Equity</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
-          <t>Consumer credit bureau in Mexico providing credit reports, scores and risk analytics to lenders</t>
+          <t>AI-powered corporate performance management (CPM) software for CFOs — financial consolidation, reporting and FP&amp;A</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr">
@@ -1009,12 +1015,12 @@
       </c>
       <c r="N8" s="7" t="inlineStr">
         <is>
-          <t>Equifax investor press release</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>LTM to 30-Jun-26 rev ~$134M (+31% YoY), adj. EBITDA ~$62M; EV $750M ($825M gross less ~$75M cash, no debt) -&gt; 5.6x rev / 12.1x EBITDA</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P8" s="4" t="inlineStr">
@@ -1042,12 +1048,12 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Financial Info &amp; Analytics</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -1062,32 +1068,26 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Send Technology Solutions</t>
+          <t>Círculo de Crédito</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Duck Creek Technologies</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K9" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Equifax</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>12.1</v>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>AI-native underwriting orchestration engine for commercial, specialty, reinsurance and MGA/delegated-authority insurers</t>
+          <t>Consumer credit bureau in Mexico providing credit reports, scores and risk analytics to lenders</t>
         </is>
       </c>
       <c r="M9" s="8" t="inlineStr">
@@ -1097,12 +1097,12 @@
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Equifax investor press release</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>LTM to 30-Jun-26 rev ~$134M (+31% YoY), adj. EBITDA ~$62M; EV $750M ($825M gross less ~$75M cash, no debt) -&gt; 5.6x rev / 12.1x EBITDA</t>
         </is>
       </c>
       <c r="P9" s="4" t="inlineStr">
@@ -1130,87 +1130,175 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
+          <t>InsurTech</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Strategic M&amp;A</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>07-Jul-26</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Send Technology Solutions</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Duck Creek Technologies</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>AI-native underwriting orchestration engine for commercial, specialty, reinsurance and MGA/delegated-authority insurers</t>
+        </is>
+      </c>
+      <c r="M10" s="8" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="N10" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P10" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R10" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>10-Jul-26</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
           <t>Payments</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Strategic M&amp;A</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>08-Jul-26</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>Cypher</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>Nium</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J10" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K10" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L10" s="7" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="inlineStr">
         <is>
           <t>Crypto-native non-custodial wallet and card-issuing platform bridging fiat and on-chain money movement</t>
         </is>
       </c>
-      <c r="M10" s="8" t="inlineStr">
+      <c r="M11" s="8" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="N10" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O10" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P10" s="4" t="inlineStr">
+      <c r="N11" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P11" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="Q10" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R10" s="4" t="inlineStr">
+      <c r="Q11" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R11" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B3:R10"/>
+  <autoFilter ref="B3:R11"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId2"/>
@@ -1219,6 +1307,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1230,7 +1319,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:M7"/>
+  <dimension ref="A3:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.73" customWidth="1" min="1" max="1"/>
@@ -1381,7 +1470,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Capital Markets Tech</t>
+          <t>Banking &amp; Lending Tech</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -1391,21 +1480,21 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>07-Jul-26</t>
+          <t>09-Jul-26</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>EDX Markets</t>
+          <t>MountainSeed</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>SBI Holdings</t>
+          <t>Long Ridge Equity Partners</t>
         </is>
       </c>
       <c r="H5" s="5" t="n">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
@@ -1424,7 +1513,7 @@
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>Institutional-only digital-asset trading venue paired with a separate central clearinghouse to reduce counterparty risk</t>
+          <t>AI-powered appraisal-management and valuation platform with capital-markets solutions for community banks and credit unions</t>
         </is>
       </c>
       <c r="M5" s="8" t="inlineStr">
@@ -1442,7 +1531,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Financial Info &amp; Analytics</t>
+          <t>Capital Markets Tech</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -1457,19 +1546,21 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Norm Ai</t>
+          <t>EDX Markets</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Khosla Ventures</t>
+          <t>SBI Holdings</t>
         </is>
       </c>
       <c r="H6" s="5" t="n">
-        <v>120</v>
-      </c>
-      <c r="I6" s="5" t="n">
-        <v>1200</v>
+        <v>76</v>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
@@ -1483,7 +1574,7 @@
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
-          <t>AI-native regulatory-compliance and legal-review platform deploying rules-trained agents for banks, insurers, asset managers and other regulated enterprises</t>
+          <t>Institutional-only digital-asset trading venue paired with a separate central clearinghouse to reduce counterparty risk</t>
         </is>
       </c>
       <c r="M6" s="8" t="inlineStr">
@@ -1501,65 +1592,251 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
+          <t>Capital Markets Tech</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>07-Jul-26</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>GoCharting</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Long Ridge Equity Partners</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>Web-native multi-asset order-flow charting and technical-analysis platform for retail and professional traders</t>
+        </is>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>10-Jul-26</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Corporate Financial Function</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>07-Jul-26</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Skello</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Bridgepoint</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>230</v>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>Workforce-scheduling and HR-management platform for frontline, shift-based teams — rostering, time-tracking and payroll preparation</t>
+        </is>
+      </c>
+      <c r="M8" s="8" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>10-Jul-26</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Financial Info &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>07-Jul-26</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Norm Ai</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Khosla Ventures</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>AI-native regulatory-compliance and legal-review platform deploying rules-trained agents for banks, insurers, asset managers and other regulated enterprises</t>
+        </is>
+      </c>
+      <c r="M9" s="8" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>10-Jul-26</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
           <t>Real Estate &amp; Mortgage Tech</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>United Kingdom</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>08-Jul-26</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>Kord</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Guinness Ventures</t>
         </is>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="H10" s="5" t="n">
         <v>8.6</v>
       </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K7" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L7" s="7" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
         <is>
           <t>FCA-regulated platform unifying identity/AML checks and client-money payment processing for estate agents, conveyancers and law firms</t>
         </is>
       </c>
-      <c r="M7" s="8" t="inlineStr">
+      <c r="M10" s="8" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M7"/>
+  <autoFilter ref="A3:M10"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>